<commit_message>
vault backup: 2026-10-13 20:18:06
</commit_message>
<xml_diff>
--- a/deploy/菲律宾部署方案-v2.3-修订版.xlsx
+++ b/deploy/菲律宾部署方案-v2.3-修订版.xlsx
@@ -15630,7 +15630,11 @@
         <f>IF(AND($G59&lt;=15,$H59&gt;=15),"■■","")</f>
         <v/>
       </c>
-      <c r="Y59" s="17" t="n"/>
+      <c r="Y59" s="17" t="inlineStr">
+        <is>
+          <t>⏸ 2026-10-13 负责人裁定：本卡挂起 · 按需再做（8 个固定 EIP 已于 Day1 任务 6/12 建成并提交上游，台账留存备用；重启触发条件＝① Day4 正式发布前确定使用的渠道中存在需上游 IP 白名单者（企业专属 / Azure OpenAI / 自建上游）、② 任一渠道稳定 403 或间歇失败且排除 SNAT/EIP 侧、③ 上游主动要求提交和回执；详见指南任务 56 卡）</t>
+        </is>
+      </c>
       <c r="Z59" s="17" t="n"/>
       <c r="AA59" s="17" t="n"/>
       <c r="AB59" s="16" t="inlineStr">
@@ -15640,7 +15644,7 @@
       </c>
       <c r="AC59" s="16" t="inlineStr">
         <is>
-          <t>未开始</t>
+          <t>⏸ 挂起 · 按需再做（2026-10-13 裁定：暂不执行，不进执行队列，不阻塞 M3）</t>
         </is>
       </c>
       <c r="AD59" s="17">

</xml_diff>

<commit_message>
docs(deploy): 登记路② 落地（2026-10-15 两地 443 出证来源反转为 Ingress spec.tls Secret）
新增 manifests/ingress-alb-tls-anchor.yaml（两地现网锚点对象副本，含四条硬约束与 apply/回滚/验收命令）；
cert/targets.yaml 补 evidence_20261015 与 target_state、新增 R5（刷 Secret 为唯一换绑通道）、把「改 AlbConfig 即够」的旧口径标注为已反转；
指南 v2.0 任务 3 卡与任务 40 前置/判据同步更正；xlsx 台账 5 格（B18/K20/K21/AC6/AC43）按同一口径修订。

诚实缺口：G1 集群内定时刷 Secret 执行器未实现（免人工尚未兑现，续签窗口仍须人工 R5）；
G2「Secret 内证书已过期时是否仍优先」未证；G3 续签后私钥是否不变未证。
</commit_message>
<xml_diff>
--- a/deploy/菲律宾部署方案-v2.3-修订版.xlsx
+++ b/deploy/菲律宾部署方案-v2.3-修订版.xlsx
@@ -1572,7 +1572,7 @@
       </c>
       <c r="B18" s="16" t="inlineStr">
         <is>
-          <t>① 工期 5 天 -&gt; 9 天（v2.0 -&gt; v2.1：56 项任务压缩进 8 天/16 时段经 600 次重排无可行解）；② 前置期 T-3 的 0 天改为真实前置 T-5；③ 补 PgBouncer/RDS 代理、cluster-autoscaler、备 region HPA 与 1.5× 接管容量；④ 补 staging/perf、运维访问面、Tair 预热、PITR 演练、连接数预算、Grafana、带宽与成本量化、上游配额盘点；⑤ 安全 3 改（ALB 源收敛为 WAF/DCDN 回源段、支付回调源 IP 白名单、SESSION_SECRET 双密钥轮换）；⑥ 修正证书部署时序、依赖倒挂、J48 负荷公式、门禁计数与编号映射、域名/数据盘/RTT 阈值口径；⑦【v2.2】工期 9 天 -&gt; 5 天：把每天 2 个半天时段改为 3 个工作段（新增 19:00–23:00 晚间加班段），15 时段 × 2 人 × 4 人时 = 120 人时产能，56 项任务在 15 段内重排完成、0 超载；⑧【v2.3】备 region 容量口径改为「本期仅承载 PH 备、不含泰国备」：节点数按 Pod requests 反算并留 ≥ 20% 系统组件余量 → 8 节点，节点池 2–12 改 2–8、配额 96 改 64 vCPU；统一「1.5×」基准为 maxReplicas × 1.5；⑨【2026-09-24 决策定案】三项遗留决策：保留 D4/D5 国庆窗口（不顺延）、T-5 = 2026-09-23 基准不动、本期不增加第 3 人。⑩【2026-10-08 按指南 v2.0（2026-10-07 版）实况回改】共回改 146 格：① 机型 g8i → g9i 首选（三机型列表，实开 g9ae）；② 主站 HPA 4–16 → 4–13、备站接管 16×1.5=24 → 13×1.5=19.5 → 20 副本；PDB minAvailable=3 → 70%；③ 新加坡配额实批按量 96 vCPU、节点池上限 12（v2.3 的 64 vCPU / 8 节点保留为容量下限）；④ RDS 规格 16C64G → pg.n4.2c.2m（2C8G，max_connections=800）；⑤ PgBouncer 自建 → RDS 内置托管池（F10 撤销）；⑥ 日志库 → 马尼拉 ClickHouse 企业版单 AZ（F9），不再购买新加坡 CK；⑦ 凭据链路 → 不使用 KMS/RRSA/ExternalSecret（2026-10-05 裁定），改手工 Opaque Secret；⑧ ECS 节点池付费方式定为按量 PostPaid（F13），成本按实况整机单价重算；⑨ 备站 Pod SQL_MAX_OPEN_CONNS=10（CM 100）；⑩ 伸缩组件实名 ack-goatscaler（非 cluster-autoscaler，观测入口 cm/kube-system/autoscaler-meta）；⑪ 任务 53 收敛口径由「30s × 节点数」改为「≤30 s（与节点数、跨 region 无关）」；⑫ 健康检查路径 /api/status 与全局限流冲突（应改 /readyz 并免限流）；⑬ 落地计划 AC 列按实况回填（21 张已完成 / 8 张部分交付 / 27 张未开始）。⑭【2026-10-12 与指南同步】：① G5 证书闭环——实购 Alibaba 品牌 DV 通配符 ali.dv.w（US$207，CertIdentifier=606823-ap-southeast-1，SAN *.likha.hk + likha.hk，链至 DigiCert Global Root G2），原 GlobalSign OV（US$997）已全额退款；⚠ 单张有效期仅 198 天（→ 2027-04-28）且 **AutoReissue=enable**（2026-10-12 经授权 UpdateInstance 开启，GetInstanceDetail 与 ListInstances 双路回读；写前 disable）⇒ 实例级托管续签已开，但不代表 443 自动续上：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」），且 ALB 是 ServiceManagedResource（直调 OpenAPI 换绑实测 3/3 被拒）⇒ 新证签发后须改 AlbConfig 再 apply（2027-03-29 前，deploy/cert/targets.yaml R1–R4；免人工的两条改法见指南任务 3 卡 ★ 段）；② 两地 ALB 443 监听 + 证书 + HTTP→HTTPS 301 已落地并验收（任务 19 V1–V5 全过、任务 25 闭合），requestTimeout 口径 180s → 600s（ALB 硬上限）；③ WAF 仍未接入（账号无实例；版本由「企业版」改为待裁定，2026-10-10 选型建议高级版）；④ GTM 仍挂起（任务 21，2026-09-30 裁定）；⑤ 备站跨区写马尼拉 CK 已实测在位（PUBLIC 端点 + sg_eip 白名单，2026-10-09 复核），原「待裁定」闭合；⑥ 任务 26 观测 4/4 闭环、任务 27 canary V1–V6 全过、任务 53 按更正判据通过；⑦ 镜像前缀按实测 EE 域名更正（B27）。⑮【2026-10-12 WAF 购买决策】：项目负责人裁定本次部署**不购买 WAF 3.0**（暂缓、非取消）——最低档高级版 3,880 元/月 ≈US$556 + 2,000 QPS + 日志服务单独起购，相对当前业务量过高，且实例只能控制台订阅（waf-openapi 无 CreateInstance、CLI 不能报价下单）。连锁更正：任务 20 整体挂起、V1–V4 从上线门禁移出；任务 47「ALB 入向不收敛」失去 WAF 缓解（443 直接暴露公网、无前置 L7 层，收敛与否重开为待裁定）；任务 40 证书部署对象只剩 ALB；任务 48 回调防线确定为两层（应用白名单 + 签名）；任务 52 成本表 WAF 行归零；M3 通过标准去掉 WAF；备站接管后同样无 L7 防护（任务 25 坑 2 转为知情接受风险）；CC 攻击的损失形态改为 HPA 按量扩容 + ALB LCU + 上游 token，故预算 80% 告警与异常突增巡检升为必须项。复评触发条件＝日请求量显著增长 / 出现真实攻击或 CC 事件。依据＝指南 §0.5 F15（2026-10-12 裁定）。</t>
+          <t>① 工期 5 天 -&gt; 9 天（v2.0 -&gt; v2.1：56 项任务压缩进 8 天/16 时段经 600 次重排无可行解）；② 前置期 T-3 的 0 天改为真实前置 T-5；③ 补 PgBouncer/RDS 代理、cluster-autoscaler、备 region HPA 与 1.5× 接管容量；④ 补 staging/perf、运维访问面、Tair 预热、PITR 演练、连接数预算、Grafana、带宽与成本量化、上游配额盘点；⑤ 安全 3 改（ALB 源收敛为 WAF/DCDN 回源段、支付回调源 IP 白名单、SESSION_SECRET 双密钥轮换）；⑥ 修正证书部署时序、依赖倒挂、J48 负荷公式、门禁计数与编号映射、域名/数据盘/RTT 阈值口径；⑦【v2.2】工期 9 天 -&gt; 5 天：把每天 2 个半天时段改为 3 个工作段（新增 19:00–23:00 晚间加班段），15 时段 × 2 人 × 4 人时 = 120 人时产能，56 项任务在 15 段内重排完成、0 超载；⑧【v2.3】备 region 容量口径改为「本期仅承载 PH 备、不含泰国备」：节点数按 Pod requests 反算并留 ≥ 20% 系统组件余量 → 8 节点，节点池 2–12 改 2–8、配额 96 改 64 vCPU；统一「1.5×」基准为 maxReplicas × 1.5；⑨【2026-09-24 决策定案】三项遗留决策：保留 D4/D5 国庆窗口（不顺延）、T-5 = 2026-09-23 基准不动、本期不增加第 3 人。⑩【2026-10-08 按指南 v2.0（2026-10-07 版）实况回改】共回改 146 格：① 机型 g8i → g9i 首选（三机型列表，实开 g9ae）；② 主站 HPA 4–16 → 4–13、备站接管 16×1.5=24 → 13×1.5=19.5 → 20 副本；PDB minAvailable=3 → 70%；③ 新加坡配额实批按量 96 vCPU、节点池上限 12（v2.3 的 64 vCPU / 8 节点保留为容量下限）；④ RDS 规格 16C64G → pg.n4.2c.2m（2C8G，max_connections=800）；⑤ PgBouncer 自建 → RDS 内置托管池（F10 撤销）；⑥ 日志库 → 马尼拉 ClickHouse 企业版单 AZ（F9），不再购买新加坡 CK；⑦ 凭据链路 → 不使用 KMS/RRSA/ExternalSecret（2026-10-05 裁定），改手工 Opaque Secret；⑧ ECS 节点池付费方式定为按量 PostPaid（F13），成本按实况整机单价重算；⑨ 备站 Pod SQL_MAX_OPEN_CONNS=10（CM 100）；⑩ 伸缩组件实名 ack-goatscaler（非 cluster-autoscaler，观测入口 cm/kube-system/autoscaler-meta）；⑪ 任务 53 收敛口径由「30s × 节点数」改为「≤30 s（与节点数、跨 region 无关）」；⑫ 健康检查路径 /api/status 与全局限流冲突（应改 /readyz 并免限流）；⑬ 落地计划 AC 列按实况回填（21 张已完成 / 8 张部分交付 / 27 张未开始）。⑭【2026-10-12 与指南同步】：① G5 证书闭环——实购 Alibaba 品牌 DV 通配符 ali.dv.w（US$207，CertIdentifier=606823-ap-southeast-1，SAN *.likha.hk + likha.hk，链至 DigiCert Global Root G2），原 GlobalSign OV（US$997）已全额退款；⚠ 单张有效期仅 198 天（→ 2027-04-28）且 **AutoReissue=enable**（2026-10-12 经授权 UpdateInstance 开启，GetInstanceDetail 与 ListInstances 双路回读；写前 disable）⇒ 实例级托管续签已开，但不代表 443 自动续上：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」），且 ALB 是 ServiceManagedResource（直调 OpenAPI 换绑实测 3/3 被拒）⇒ ★ 2026-10-15 路② 已落地两地（Secret/new-api-tls + 锚定 Ingress new-api-tls-anchor），443 同域名出证来源 = Ingress spec.tls 的 Secret（实测压住 AlbConfig 钉死证，钉死证保留未撤）⇒ 新证签发后必须**刷 Secret**（deploy/cert/targets.yaml R5 = 必需路径），只改 AlbConfig 不再足以恢复 443（2027-03-29 前，targets.yaml R1–R5；机制取证与落地验收见指南任务 3 卡 ★ 段）。⚠ 刷 Secret 的执行器尚未实现 ⇒ 现阶段续签仍需人工；② 两地 ALB 443 监听 + 证书 + HTTP→HTTPS 301 已落地并验收（任务 19 V1–V5 全过、任务 25 闭合），requestTimeout 口径 180s → 600s（ALB 硬上限）；③ WAF 仍未接入（账号无实例；版本由「企业版」改为待裁定，2026-10-10 选型建议高级版）；④ GTM 仍挂起（任务 21，2026-09-30 裁定）；⑤ 备站跨区写马尼拉 CK 已实测在位（PUBLIC 端点 + sg_eip 白名单，2026-10-09 复核），原「待裁定」闭合；⑥ 任务 26 观测 4/4 闭环、任务 27 canary V1–V6 全过、任务 53 按更正判据通过；⑦ 镜像前缀按实测 EE 域名更正（B27）。⑮【2026-10-12 WAF 购买决策】：项目负责人裁定本次部署**不购买 WAF 3.0**（暂缓、非取消）——最低档高级版 3,880 元/月 ≈US$556 + 2,000 QPS + 日志服务单独起购，相对当前业务量过高，且实例只能控制台订阅（waf-openapi 无 CreateInstance、CLI 不能报价下单）。连锁更正：任务 20 整体挂起、V1–V4 从上线门禁移出；任务 47「ALB 入向不收敛」失去 WAF 缓解（443 直接暴露公网、无前置 L7 层，收敛与否重开为待裁定）；任务 40 证书部署对象只剩 ALB；任务 48 回调防线确定为两层（应用白名单 + 签名）；任务 52 成本表 WAF 行归零；M3 通过标准去掉 WAF；备站接管后同样无 L7 防护（任务 25 坑 2 转为知情接受风险）；CC 攻击的损失形态改为 HPA 按量扩容 + ALB LCU + 上游 token，故预算 80% 告警与异常突增巡检升为必须项。复评触发条件＝日请求量显著增长 / 出现真实攻击或 CC 事件。依据＝指南 §0.5 F15（2026-10-12 裁定）。</t>
         </is>
       </c>
     </row>
@@ -2873,7 +2873,7 @@
       </c>
       <c r="K20" s="36" t="inlineStr">
         <is>
-          <t>私钥**不落 KMS**（2026-10-05 裁定不使用 KMS/凭据管家）：证书私钥由运维手工保管；⚠ 2026-10-12 实况：单张有效期仅 198 天（→ 2027-04-28，CA/B 新规）；AutoReissue=enable（2026-10-12 经授权开启并双路回读）⇒ 实例级托管续签已开，但不代表 443 自动续上：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」），且 ALB 是 ServiceManagedResource（直调 OpenAPI 换绑实测 3/3 被拒）⇒ 新证签发后须改 AlbConfig 再 apply（2027-03-29 前，deploy/cert/targets.yaml R1–R4；免人工的两条改法见指南任务 3 卡 ★ 段）；30 天到期告警已在控制台配置（2026-10-12 负责人自配；⚠ CAS 无提醒类 API，故该项无回读证据、配置页截图待补）</t>
+          <t>私钥**不落 KMS**（2026-10-05 裁定不使用 KMS/凭据管家）：证书私钥由运维手工保管；⚠ 2026-10-12 实况：单张有效期仅 198 天（→ 2027-04-28，CA/B 新规）；AutoReissue=enable（2026-10-12 经授权开启并双路回读）⇒ 实例级托管续签已开，但不代表 443 自动续上：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」），且 ALB 是 ServiceManagedResource（直调 OpenAPI 换绑实测 3/3 被拒）⇒ ★ 2026-10-15 路② 已落地两地（Secret/new-api-tls + 锚定 Ingress new-api-tls-anchor），443 同域名出证来源 = Ingress spec.tls 的 Secret（实测压住 AlbConfig 钉死证，钉死证保留未撤）⇒ 新证签发后必须**刷 Secret**（deploy/cert/targets.yaml R5 = 必需路径），只改 AlbConfig 不再足以恢复 443（2027-03-29 前，targets.yaml R1–R5；机制取证与落地验收见指南任务 3 卡 ★ 段）。⚠ 刷 Secret 的执行器尚未实现 ⇒ 现阶段续签仍需人工；30 天到期告警已在控制台配置（2026-10-12 负责人自配；⚠ CAS 无提醒类 API，故该项无回读证据、配置页截图待补）</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="K21" s="38" t="inlineStr">
         <is>
-          <t>⚠ 2026-10-12 更正：AutoReissue=enable（2026-10-12 经授权开启，GetInstanceDetail/ListInstances 双路回读）⇒ 实例级托管续签已开，但监听只认 AlbConfig 钉死的 CertificateId（且 ALB 为 ServiceManagedResource，直调 OpenAPI 换绑被拒）⇒ 新证书签发后须改 AlbConfig 再 apply 并回归验证（到期 2027-04-28，动作 2027-03-29 前）</t>
+          <t>⚠ 2026-10-12 更正：AutoReissue=enable（2026-10-12 经授权开启，GetInstanceDetail/ListInstances 双路回读）⇒ 实例级托管续签已开，但监听只认 AlbConfig 钉死的 CertificateId（且 ALB 为 ServiceManagedResource，直调 OpenAPI 换绑被拒）⇒ ★ 2026-10-15 路② 已落地：443 出证来源改为 Ingress spec.tls 的 Secret（同域名压住 AlbConfig 钉死证，已实测）⇒ 新证书签发后须刷两地 TLS Secret（targets.yaml R5）并回归验证（到期 2027-04-28，动作 2027-03-29 前）；只改 AlbConfig 不再足以换绑，刷 Secret 的执行器尚未实现 ⇒ 现阶段仍需人工</t>
         </is>
       </c>
     </row>
@@ -9545,7 +9545,7 @@
       </c>
       <c r="AC6" s="16" t="inlineStr">
         <is>
-          <t>已完成（2026-10-12 实测 4/4 交付，本卡闭合）：① 私钥+全链入 /root/.deploy_secrets/TLS_WILDCARD_{CRT,KEY}（-rw------- root root 6075/1675、leaf 在前、链 3 张、-modulus md5 两侧同为 df343b79775… ⇒ 配对 PASS，执行器 deploy/logs/tls_store_20261012.sh）；② notAfter=2027-04-28 ≥ 今+30 天、SAN 含 *.likha.hk 与 likha.hk、openssl verify OK、CAS CertificateStatus=issued（CertId=606823）；③ 到期告警：控制台由负责人自配（⚠ 无 API 可取证，证据=负责人确认，配置页截图仍欠），另经授权开实例级自动托管续签 UpdateInstance --AutoReissue enable，GetInstanceDetail 与 ListInstances 双路回读均为 enable（写前 disable）；④ 模板落地 deploy/cert/targets.yaml（含现场回读的 ALB/监听 ID）。★ 长期风险如实登记（2026-10-12 二次取证订正）：AutoReissueCount 仍 0、ListTrusteeOrder NotFound；早前据 ListCloudResources --CloudName alb 的 Total=0 判「CAS 无部署联动」是**参数用错的假阴性**（--CloudName 是云厂商，ALB 属 --CloudProduct；正确调用实测到两地监听已在 CAS 登记 Id=37274711/37274712，但那是资源可见性、不是"托管会自动写入"）。真实结论由控制面语义决定：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」；两地实测各只绑 1 张、无多证书兜底），而 ALB 是 ServiceManagedResource（直调 UpdateListenerAttribute 实测 3/3 被拒）⇒ 换绑的唯一通道是**改 AlbConfig 再 apply**（R1–R4 已按此订正，2027-03-29 前执行）。免人工改法（双证共存 / Secret 自动触发）与两条未证风险见指南任务 3 卡 ★ 段。⚠ 另：本轮调试用 bash -x 把私钥正文留在本机会话记录（无远端副本），负责人裁定按「接受」处置，2027-03 续签窗口自然换新；永久规则=处理私钥的脚本禁 -x。</t>
+          <t>已完成（2026-10-12 实测 4/4 交付，本卡闭合）：① 私钥+全链入 /root/.deploy_secrets/TLS_WILDCARD_{CRT,KEY}（-rw------- root root 6075/1675、leaf 在前、链 3 张、-modulus md5 两侧同为 df343b79775… ⇒ 配对 PASS，执行器 deploy/logs/tls_store_20261012.sh）；② notAfter=2027-04-28 ≥ 今+30 天、SAN 含 *.likha.hk 与 likha.hk、openssl verify OK、CAS CertificateStatus=issued（CertId=606823）；③ 到期告警：控制台由负责人自配（⚠ 无 API 可取证，证据=负责人确认，配置页截图仍欠），另经授权开实例级自动托管续签 UpdateInstance --AutoReissue enable，GetInstanceDetail 与 ListInstances 双路回读均为 enable（写前 disable）；④ 模板落地 deploy/cert/targets.yaml（含现场回读的 ALB/监听 ID）。★ 长期风险如实登记（2026-10-12 二次取证订正）：AutoReissueCount 仍 0、ListTrusteeOrder NotFound；早前据 ListCloudResources --CloudName alb 的 Total=0 判「CAS 无部署联动」是**参数用错的假阴性**（--CloudName 是云厂商，ALB 属 --CloudProduct；正确调用实测到两地监听已在 CAS 登记 Id=37274711/37274712，但那是资源可见性、不是"托管会自动写入"）。真实结论由控制面语义决定：监听只认 AlbConfig 钉死的 CertificateId（ACK 原文「Listener 不会使用自动发现证书，优先使用 AlbConfig 指定的证书」；两地实测各只绑 1 张、无多证书兜底），而 ALB 是 ServiceManagedResource（直调 UpdateListenerAttribute 实测 3/3 被拒）⇒ 当时的换绑通道是**改 AlbConfig 再 apply**（R1–R4 已按此订正）。★ 2026-10-15 路② 落地两地，该"唯一通道"口径**反转**：两地各建 Secret/new-api-tls（生产真证进 etcd）+ 锚定 Ingress new-api-tls-anchor（deploy/manifests/ingress-alb-tls-anchor.yaml，只承载 spec.tls、host 无 DNS 记录），实测同域名出证来源 = Secret ⇒ **续签必须刷 Secret**（targets.yaml 新增 R5 = 必需路径），只改 AlbConfig 不再足以恢复 443。验收（回写前重跑复现）：两地 cert_count=2（Secret 证 IsDefault=false + 钉死证仍 true）、SNI 10/10 serial 与基线逐字一致（换来源不换证书）、业务码不变、sg 原 4 条 RuleId 逐字未动、既有业务 Ingress rv 全未变。⚠ 未兑现：刷 Secret 的执行器尚未实现（G1）⇒ 现阶段续签仍需人工；「Secret 证已过期时是否仍优先」（G2）与「续签后私钥是否不变」（G3）未证。落地通道＝甲（ECS RunCommand 下发；正文可被 ActionTrail 留存 90 天与 DescribeInvocations 回读），属一次性放行，常态化需再裁定。⚠ 另：本轮调试用 bash -x 把私钥正文留在本机会话记录（无远端副本），负责人裁定按「接受」处置，2027-03 续签窗口自然换新；永久规则=处理私钥的脚本禁 -x。</t>
         </is>
       </c>
       <c r="AD6" s="17">
@@ -13800,7 +13800,7 @@
       </c>
       <c r="AC43" s="16" t="inlineStr">
         <is>
-          <t>部分交付（2026-10-12：证书已部署至两地 ALB 443，链校验与 SNI 通过；WAF 未接入、DCDN 未启用 ⇒ 按 F15（不采购）与未开通，本轮不做，判据收窄为仅 ALB；未闭合项改为「新证书须改 AlbConfig 再 apply 才会换绑（AutoReissue=enable 只保证 CAS 签出新证；ALB 为 ServiceManagedResource，直调 OpenAPI 被拒；2027-03-29 前执行 targets.yaml R1–R4）」）</t>
+          <t>部分交付（2026-10-12：证书已部署至两地 ALB 443，链校验与 SNI 通过；WAF 未接入、DCDN 未启用 ⇒ 按 F15（不采购）与未开通，本轮不做，判据收窄为仅 ALB；未闭合项（2026-10-15 更新）「新证书须**刷两地 TLS Secret**（targets.yaml R5）才会换绑 —— 路② 已落地、443 出证来源 = Secret；AutoReissue=enable 只保证 CAS 签出新证，ALB 为 ServiceManagedResource 直调 OpenAPI 被拒，改 AlbConfig（R2）已降为次要动作；2027-03-29 前执行 targets.yaml R1–R5」）</t>
         </is>
       </c>
       <c r="AD43" s="17">

</xml_diff>